<commit_message>
Evidencia final del despliegue (20/20) y comparación fija contra el commit anterior
- verificar-despliegue.mjs: JEN-03 diagnostica el último build no exitoso (#12, Quality Gate sin
  cobertura) y JEN-04 reutiliza el build existente sobre el commit HEAD o lo dispara y espera.
- Build #13 de Jenkins sobre Andres-Arango280/task_flow: SUCCESS, Quality Gate OK, 137 pruebas.
- comparar.mjs: la versión anterior es siempre el commit 8b46dc0 (REF_ANTES), no HEAD.
- README_RUBRICA.md, matriz, plan, informe y presentación regenerados.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pruebas/evidencias/matriz/Matriz-Trazabilidad-TaskFlow.xlsx
+++ b/pruebas/evidencias/matriz/Matriz-Trazabilidad-TaskFlow.xlsx
@@ -5872,7 +5872,7 @@
     <t>Quality Gate del backend</t>
   </si>
   <si>
-    <t>Quality Gate=OK; condiciones: new_reliability_rating OK (1 vs GT 1) · new_security_rating OK (1 vs GT 1) · new_maintainability_rating OK (1 vs GT 1) · new_coverage OK (87.1 vs LT 80) · new_duplicated_lines_density OK (0.0 vs GT 3) · new_security_hotspots_reviewed OK (100.0 vs LT 100). bugs=0, vulnerabilidades=0, code smells=1, cobertura=87.2 %, duplicación=0.0 %, hotspots=0, ncloc=866; análisis registrados=5</t>
+    <t>Quality Gate=OK; condiciones: new_reliability_rating OK (1 vs GT 1) · new_security_rating OK (1 vs GT 1) · new_maintainability_rating OK (1 vs GT 1) · new_coverage OK (88.1 vs LT 80) · new_duplicated_lines_density OK (0.0 vs GT 3) · new_security_hotspots_reviewed OK (100.0 vs LT 100). bugs=0, vulnerabilidades=0, code smells=1, cobertura=87.2 %, duplicación=0.0 %, hotspots=0, ncloc=866; análisis registrados=9</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/despliegue/sonar/backend-quality-gate.json
@@ -5898,7 +5898,7 @@
     <t>Quality Gate del frontend</t>
   </si>
   <si>
-    <t>Quality Gate=OK; condiciones: new_reliability_rating OK (1 vs GT 1) · new_security_rating OK (1 vs GT 1) · new_maintainability_rating OK (1 vs GT 1). bugs=0, vulnerabilidades=0, code smells=0, cobertura=— %, duplicación=0.0 %, hotspots=0, ncloc=264; análisis registrados=2</t>
+    <t>Quality Gate=OK; condiciones: new_reliability_rating OK (1 vs GT 1) · new_security_rating OK (1 vs GT 1) · new_maintainability_rating OK (1 vs GT 1) · new_duplicated_lines_density OK (0.0 vs GT 3). bugs=0, vulnerabilidades=0, code smells=0, cobertura=— %, duplicación=0.0 %, hotspots=0, ncloc=264; análisis registrados=4</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/despliegue/sonar/frontend-quality-gate.json
@@ -5912,7 +5912,7 @@
     <t>Servidor Jenkins y job del pipeline disponibles</t>
   </si>
   <si>
-    <t>Jenkins OK (1 jobs); taskflow-pipeline: color=red, último build #11 (FAILURE), último exitoso #10</t>
+    <t>Jenkins OK (1 jobs); taskflow-pipeline: color=blue, último build #13 (SUCCESS), último exitoso #13</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/despliegue/jenkins/jenkins-api.json
@@ -5922,35 +5922,35 @@
     <t>JEN-02</t>
   </si>
   <si>
-    <t>Último build exitoso del pipeline (#10)</t>
-  </si>
-  <si>
-    <t>Build #10 del 23/9/2026, 10:37:44 p. m. sobre el commit 8b46dc0: etapas Declarative: Checkout SCM → Declarative: Tool Install → Checkout → Instalar dependencias → Ejecutar pruebas unitarias → Compilar aplicación → Analisis con SonarQube → Quality Gate → Construir imagen Docker → Declarative: Post Actions; Tests:       35 passed, 35 total; Quality Gate OK; resultado SUCCESS.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pruebas/evidencias/despliegue/jenkins/build-10-consola.log
+    <t>Último build exitoso del pipeline (#13)</t>
+  </si>
+  <si>
+    <t>Build #13 del 27/10/2026, 12:21:27 a. m. sobre el commit f6522aa: etapas Declarative: Checkout SCM → Declarative: Tool Install → Checkout → Instalar dependencias → Pruebas de regresión unitarias → Pruebas de regresión caja negra → Compilar aplicación → Analisis con SonarQube → Quality Gate → Construir imagen Docker → Declarative: Post Actions; Tests:       88 passed, 88 total | Tests:       49 passed, 49 total; Quality Gate OK; resultado SUCCESS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pruebas/evidencias/despliegue/jenkins/build-13-consola.log
 pruebas/evidencias/despliegue/jenkins/job-api.json</t>
   </si>
   <si>
     <t>JEN-03</t>
   </si>
   <si>
-    <t>Diagnóstico del último build (#11, FAILURE)</t>
-  </si>
-  <si>
-    <t>Build #11: fatal: unable to access 'https://github.com/Claudia280-girl/validacion/': Could not resolve host: github.com</t>
-  </si>
-  <si>
-    <t>pruebas/evidencias/despliegue/jenkins/build-11-consola.log</t>
+    <t>Diagnóstico del último build no exitoso (#12, FAILURE)</t>
+  </si>
+  <si>
+    <t>Build #12 del 27/10/2026, 12:11:07 a. m.: QUALITY GATE STATUS: FAILED - View details on http://sonarqube:9000/dashboard?id=taskflow%3Abackend — el análisis se ejecutó sin coverage/lcov.info (sensor de cobertura cero → new_coverage 0 %).</t>
+  </si>
+  <si>
+    <t>pruebas/evidencias/despliegue/jenkins/build-12-consola.log</t>
   </si>
   <si>
     <t>JEN-04</t>
   </si>
   <si>
-    <t>Nuevo build del pipeline sobre la versión refactorizada</t>
-  </si>
-  <si>
-    <t>Pendiente: 1) git add -A &amp;&amp; git commit &amp;&amp; git push origin main; 2) defina JENKINS_USER y JENKINS_TOKEN (Jenkins → usuario → Configurar → API Token) y vuelva a ejecutar este script, o pulse «Construir ahora» en http://localhost:8081/job/taskflow-pipeline y guarde la consola en pruebas/evidencias/despliegue/jenkins/.</t>
+    <t>Build final del pipeline sobre la versión refactorizada (#13)</t>
+  </si>
+  <si>
+    <t>Build #13 (existente) del 27/10/2026, 12:21:27 a. m. sobre el commit f6522aa: SUCCESS en 187 s; etapas Declarative: Checkout SCM → Declarative: Tool Install → Checkout → Instalar dependencias → Pruebas de regresión unitarias → Pruebas de regresión caja negra → Compilar aplicación → Analisis con SonarQube → Quality Gate → Construir imagen Docker → Declarative: Post Actions; Tests: 88 passed, 88 total | Tests: 49 passed, 49 total; Quality Gate OK.</t>
   </si>
   <si>
     <t>—</t>
@@ -6541,7 +6541,7 @@
     <t>Docker Compose (SonarQube 9.9 Community, PostgreSQL 15, Jenkins LTS), sonar-scanner, nest build, vite build, docker build</t>
   </si>
   <si>
-    <t>26/10/2026, 11:52:37 p. m.</t>
+    <t>27/10/2026, 12:31:19 a. m.</t>
   </si>
   <si>
     <t>pruebas/evidencias/despliegue/</t>
@@ -27142,14 +27142,14 @@
       <c r="H523" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I523" s="5" t="s">
-        <v>1427</v>
+      <c r="I523" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="J523" s="2" t="s">
         <v>1812</v>
       </c>
       <c r="K523" s="2" t="s">
-        <v>23</v>
+        <v>1805</v>
       </c>
       <c r="L523" s="2" t="s">
         <v>23</v>
@@ -28337,13 +28337,13 @@
         <v>13</v>
       </c>
       <c r="F24" s="2">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G24" s="2">
         <v>0</v>
       </c>
       <c r="H24" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>1927</v>
@@ -28565,7 +28565,7 @@
         <v>55</v>
       </c>
       <c r="G5" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H5" s="2">
         <v>0</v>
@@ -29080,13 +29080,13 @@
         <v>20</v>
       </c>
       <c r="E14">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F14">
         <v>0</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" t="s">
         <v>2009</v>

</xml_diff>

<commit_message>
Features Gherkin en el formato de la Clase 19 (Feature/Rule/Scenario con Given/When/Then)
- Los cuatro .feature usan palabras clave en inglés y texto en español, descripción
  Necesidad → Regla → Ejemplos, bloques Rule, el actor nombrado en el primer paso y después
  el pronombre («When ella…», «Then ella observa…»), tablas de datos en los Then, un
  Scenario Outline con Examples etiquetados @GH-03/@GH-04 y etiquetas @web/@api/@smoke.
- Definiciones de pasos adaptadas (actorDe resuelve el pronombre al actor en escena,
  DataTable para miembros, columnas y tareas); el id del caso se lee de la etiqueta @GH-xx.
- 12/12 escenarios y 106 pasos aprobados; evidencias, matriz, RTM, informe, presentación y
  READMEs regenerados.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pruebas/evidencias/matriz/Matriz-Trazabilidad-TaskFlow.xlsx
+++ b/pruebas/evidencias/matriz/Matriz-Trazabilidad-TaskFlow.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6832" uniqueCount="2112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6832" uniqueCount="2119">
   <si>
     <t>Requisito(s)</t>
   </si>
@@ -5123,10 +5123,13 @@
     <t>GH-01</t>
   </si>
   <si>
+    <t>Registro e inicio de sesión correctos</t>
+  </si>
+  <si>
     <t>E2E Gherkin + Screenplay (Cucumber)</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 9 pasos (5 de ellos de verificación «Entonces») en 3.7 s.</t>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 9 pasos (5 de ellos de verificación «Entonces») en 2.8 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-01.png
@@ -5138,7 +5141,10 @@
     <t>GH-02</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 5 pasos (2 de ellos de verificación «Entonces») en 1.7 s.</t>
+    <t>Registro con un correo ya existente</t>
+  </si>
+  <si>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 5 pasos (2 de ellos de verificación «Entonces») en 1.4 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-02.png
@@ -5150,13 +5156,13 @@
     <t>GH-03</t>
   </si>
   <si>
-    <t>Inicio de sesión rechazado con una contraseña incorrecta</t>
+    <t>Inicio de sesión rechazado</t>
   </si>
   <si>
     <t>error</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 6 pasos (3 de ellos de verificación «Entonces») en 1.7 s.</t>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 6 pasos (3 de ellos de verificación «Entonces») en 1.1 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-03.png
@@ -5168,10 +5174,7 @@
     <t>GH-04</t>
   </si>
   <si>
-    <t>Inicio de sesión rechazado con un correo que no existe</t>
-  </si>
-  <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 6 pasos (3 de ellos de verificación «Entonces») en 1.6 s.</t>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 6 pasos (3 de ellos de verificación «Entonces») en 1 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-04.png
@@ -5183,7 +5186,7 @@
     <t>GH-05</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 8 pasos (4 de ellos de verificación «Entonces») en 1.8 s.</t>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 8 pasos (4 de ellos de verificación «Entonces») en 1.4 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-05.png
@@ -5195,7 +5198,10 @@
     <t>GH-06</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 11 pasos (5 de ellos de verificación «Entonces») en 4.8 s.</t>
+    <t>Crear un equipo e invitar a un miembro registrado</t>
+  </si>
+  <si>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 11 pasos (5 de ellos de verificación «Entonces») en 3.8 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-06.png
@@ -5207,7 +5213,10 @@
     <t>GH-07</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 7 pasos (2 de ellos de verificación «Entonces») en 3.8 s.</t>
+    <t>Invitar un correo que no está registrado</t>
+  </si>
+  <si>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 7 pasos (2 de ellos de verificación «Entonces») en 2.2 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-07.png
@@ -5219,7 +5228,10 @@
     <t>GH-08</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 10 pasos (4 de ellos de verificación «Entonces») en 6.8 s.</t>
+    <t>Crear un proyecto genera un tablero con las columnas por defecto</t>
+  </si>
+  <si>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 10 pasos (4 de ellos de verificación «Entonces») en 2.8 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-08.png
@@ -5231,7 +5243,10 @@
     <t>GH-09</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 14 pasos (6 de ellos de verificación «Entonces») en 9.2 s.</t>
+    <t>Crear tareas y mover una a Hecho</t>
+  </si>
+  <si>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 14 pasos (6 de ellos de verificación «Entonces») en 7.9 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-09.png
@@ -5243,7 +5258,10 @@
     <t>GH-10</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 7 pasos (2 de ellos de verificación «Entonces») en 3.2 s.</t>
+    <t>Crear una tarea sin título</t>
+  </si>
+  <si>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 7 pasos (2 de ellos de verificación «Entonces») en 2.5 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-10.png
@@ -5255,7 +5273,10 @@
     <t>GH-11</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 12 pasos (4 de ellos de verificación «Entonces») en 5.4 s.</t>
+    <t>Eliminar una tarea y deshacer la eliminación</t>
+  </si>
+  <si>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 12 pasos (4 de ellos de verificación «Entonces») en 3.8 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-11.png
@@ -5270,7 +5291,7 @@
     <t>Una usuaria ajena al equipo no puede ver el tablero de Ana</t>
   </si>
   <si>
-    <t>Conforme a lo esperado. Se ejecutaron y superaron los 11 pasos (5 de ellos de verificación «Entonces») en 3.9 s.</t>
+    <t>Conforme a lo esperado. Se ejecutaron y superaron los 11 pasos (5 de ellos de verificación «Entonces») en 2.9 s.</t>
   </si>
   <si>
     <t xml:space="preserve">pruebas/evidencias/gherkin/capturas/GH-12.png
@@ -6487,7 +6508,7 @@
     <t>Cucumber 11.3.0 + Serenity/JS 3.48.2 (@serenity-js/cucumber) + Playwright 1.63.0</t>
   </si>
   <si>
-    <t>26/10/2026, 6:16:15 p. m.</t>
+    <t>27/10/2026, 8:38:49 a. m.</t>
   </si>
   <si>
     <t>pruebas/evidencias/gherkin/</t>
@@ -24661,10 +24682,10 @@
         <v>1580</v>
       </c>
       <c r="E458" s="2" t="s">
-        <v>1505</v>
+        <v>1581</v>
       </c>
       <c r="F458" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G458" s="2" t="s">
         <v>1507</v>
@@ -24676,10 +24697,10 @@
         <v>20</v>
       </c>
       <c r="J458" s="2" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="K458" s="2" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="L458" s="2" t="s">
         <v>23</v>
@@ -24696,13 +24717,13 @@
         <v>14</v>
       </c>
       <c r="D459" s="2" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
       <c r="E459" s="2" t="s">
-        <v>1512</v>
+        <v>1586</v>
       </c>
       <c r="F459" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G459" s="2" t="s">
         <v>1507</v>
@@ -24714,10 +24735,10 @@
         <v>20</v>
       </c>
       <c r="J459" s="2" t="s">
-        <v>1585</v>
+        <v>1587</v>
       </c>
       <c r="K459" s="2" t="s">
-        <v>1586</v>
+        <v>1588</v>
       </c>
       <c r="L459" s="2" t="s">
         <v>23</v>
@@ -24734,28 +24755,28 @@
         <v>14</v>
       </c>
       <c r="D460" s="2" t="s">
-        <v>1587</v>
+        <v>1589</v>
       </c>
       <c r="E460" s="2" t="s">
-        <v>1588</v>
+        <v>1590</v>
       </c>
       <c r="F460" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G460" s="2" t="s">
         <v>1507</v>
       </c>
       <c r="H460" s="2" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="I460" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J460" s="2" t="s">
-        <v>1590</v>
+        <v>1592</v>
       </c>
       <c r="K460" s="2" t="s">
-        <v>1591</v>
+        <v>1593</v>
       </c>
       <c r="L460" s="2" t="s">
         <v>23</v>
@@ -24772,28 +24793,28 @@
         <v>14</v>
       </c>
       <c r="D461" s="2" t="s">
-        <v>1592</v>
+        <v>1594</v>
       </c>
       <c r="E461" s="2" t="s">
-        <v>1593</v>
+        <v>1590</v>
       </c>
       <c r="F461" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G461" s="2" t="s">
         <v>1507</v>
       </c>
       <c r="H461" s="2" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="I461" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J461" s="2" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
       <c r="K461" s="2" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
       <c r="L461" s="2" t="s">
         <v>23</v>
@@ -24810,28 +24831,28 @@
         <v>14</v>
       </c>
       <c r="D462" s="2" t="s">
-        <v>1596</v>
+        <v>1597</v>
       </c>
       <c r="E462" s="2" t="s">
         <v>1525</v>
       </c>
       <c r="F462" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G462" s="2" t="s">
         <v>1507</v>
       </c>
       <c r="H462" s="2" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="I462" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J462" s="2" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="K462" s="2" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
       <c r="L462" s="2" t="s">
         <v>23</v>
@@ -24848,13 +24869,13 @@
         <v>14</v>
       </c>
       <c r="D463" s="2" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="E463" s="2" t="s">
-        <v>1533</v>
+        <v>1601</v>
       </c>
       <c r="F463" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G463" s="2" t="s">
         <v>1507</v>
@@ -24866,10 +24887,10 @@
         <v>20</v>
       </c>
       <c r="J463" s="2" t="s">
-        <v>1600</v>
+        <v>1602</v>
       </c>
       <c r="K463" s="2" t="s">
-        <v>1601</v>
+        <v>1603</v>
       </c>
       <c r="L463" s="2" t="s">
         <v>23</v>
@@ -24886,13 +24907,13 @@
         <v>14</v>
       </c>
       <c r="D464" s="2" t="s">
-        <v>1602</v>
+        <v>1604</v>
       </c>
       <c r="E464" s="2" t="s">
-        <v>1537</v>
+        <v>1605</v>
       </c>
       <c r="F464" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G464" s="2" t="s">
         <v>1507</v>
@@ -24904,10 +24925,10 @@
         <v>20</v>
       </c>
       <c r="J464" s="2" t="s">
-        <v>1603</v>
+        <v>1606</v>
       </c>
       <c r="K464" s="2" t="s">
-        <v>1604</v>
+        <v>1607</v>
       </c>
       <c r="L464" s="2" t="s">
         <v>23</v>
@@ -24924,13 +24945,13 @@
         <v>14</v>
       </c>
       <c r="D465" s="2" t="s">
-        <v>1605</v>
+        <v>1608</v>
       </c>
       <c r="E465" s="2" t="s">
-        <v>1541</v>
+        <v>1609</v>
       </c>
       <c r="F465" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G465" s="2" t="s">
         <v>1507</v>
@@ -24942,10 +24963,10 @@
         <v>20</v>
       </c>
       <c r="J465" s="2" t="s">
-        <v>1606</v>
+        <v>1610</v>
       </c>
       <c r="K465" s="2" t="s">
-        <v>1607</v>
+        <v>1611</v>
       </c>
       <c r="L465" s="2" t="s">
         <v>23</v>
@@ -24962,13 +24983,13 @@
         <v>14</v>
       </c>
       <c r="D466" s="2" t="s">
-        <v>1608</v>
+        <v>1612</v>
       </c>
       <c r="E466" s="2" t="s">
-        <v>1549</v>
+        <v>1613</v>
       </c>
       <c r="F466" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G466" s="2" t="s">
         <v>1507</v>
@@ -24980,10 +25001,10 @@
         <v>20</v>
       </c>
       <c r="J466" s="2" t="s">
-        <v>1609</v>
+        <v>1614</v>
       </c>
       <c r="K466" s="2" t="s">
-        <v>1610</v>
+        <v>1615</v>
       </c>
       <c r="L466" s="2" t="s">
         <v>23</v>
@@ -25000,28 +25021,28 @@
         <v>14</v>
       </c>
       <c r="D467" s="2" t="s">
-        <v>1611</v>
+        <v>1616</v>
       </c>
       <c r="E467" s="2" t="s">
-        <v>1553</v>
+        <v>1617</v>
       </c>
       <c r="F467" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G467" s="2" t="s">
         <v>1507</v>
       </c>
       <c r="H467" s="2" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="I467" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J467" s="2" t="s">
-        <v>1612</v>
+        <v>1618</v>
       </c>
       <c r="K467" s="2" t="s">
-        <v>1613</v>
+        <v>1619</v>
       </c>
       <c r="L467" s="2" t="s">
         <v>23</v>
@@ -25038,13 +25059,13 @@
         <v>14</v>
       </c>
       <c r="D468" s="2" t="s">
-        <v>1614</v>
+        <v>1620</v>
       </c>
       <c r="E468" s="2" t="s">
-        <v>626</v>
+        <v>1621</v>
       </c>
       <c r="F468" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G468" s="2" t="s">
         <v>1507</v>
@@ -25056,10 +25077,10 @@
         <v>20</v>
       </c>
       <c r="J468" s="2" t="s">
-        <v>1615</v>
+        <v>1622</v>
       </c>
       <c r="K468" s="2" t="s">
-        <v>1616</v>
+        <v>1623</v>
       </c>
       <c r="L468" s="2" t="s">
         <v>23</v>
@@ -25076,28 +25097,28 @@
         <v>14</v>
       </c>
       <c r="D469" s="2" t="s">
-        <v>1617</v>
+        <v>1624</v>
       </c>
       <c r="E469" s="2" t="s">
-        <v>1618</v>
+        <v>1625</v>
       </c>
       <c r="F469" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="G469" s="2" t="s">
         <v>1507</v>
       </c>
       <c r="H469" s="2" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="I469" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J469" s="2" t="s">
-        <v>1619</v>
+        <v>1626</v>
       </c>
       <c r="K469" s="2" t="s">
-        <v>1620</v>
+        <v>1627</v>
       </c>
       <c r="L469" s="2" t="s">
         <v>23</v>
@@ -25114,16 +25135,16 @@
         <v>14</v>
       </c>
       <c r="D470" s="2" t="s">
-        <v>1621</v>
+        <v>1628</v>
       </c>
       <c r="E470" s="2" t="s">
-        <v>1622</v>
+        <v>1629</v>
       </c>
       <c r="F470" s="2" t="s">
-        <v>1623</v>
+        <v>1630</v>
       </c>
       <c r="G470" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H470" s="2" t="s">
         <v>1508</v>
@@ -25132,10 +25153,10 @@
         <v>942</v>
       </c>
       <c r="J470" s="2" t="s">
-        <v>1625</v>
+        <v>1632</v>
       </c>
       <c r="K470" s="2" t="s">
-        <v>1626</v>
+        <v>1633</v>
       </c>
       <c r="L470" s="2" t="s">
         <v>23</v>
@@ -25152,16 +25173,16 @@
         <v>14</v>
       </c>
       <c r="D471" s="2" t="s">
-        <v>1627</v>
+        <v>1634</v>
       </c>
       <c r="E471" s="2" t="s">
-        <v>1628</v>
+        <v>1635</v>
       </c>
       <c r="F471" s="2" t="s">
-        <v>1623</v>
+        <v>1630</v>
       </c>
       <c r="G471" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H471" s="2" t="s">
         <v>1508</v>
@@ -25170,10 +25191,10 @@
         <v>20</v>
       </c>
       <c r="J471" s="2" t="s">
-        <v>1629</v>
+        <v>1636</v>
       </c>
       <c r="K471" s="2" t="s">
-        <v>1630</v>
+        <v>1637</v>
       </c>
       <c r="L471" s="2" t="s">
         <v>23</v>
@@ -25190,16 +25211,16 @@
         <v>14</v>
       </c>
       <c r="D472" s="2" t="s">
+        <v>1638</v>
+      </c>
+      <c r="E472" s="2" t="s">
+        <v>1639</v>
+      </c>
+      <c r="F472" s="2" t="s">
+        <v>1630</v>
+      </c>
+      <c r="G472" s="2" t="s">
         <v>1631</v>
-      </c>
-      <c r="E472" s="2" t="s">
-        <v>1632</v>
-      </c>
-      <c r="F472" s="2" t="s">
-        <v>1623</v>
-      </c>
-      <c r="G472" s="2" t="s">
-        <v>1624</v>
       </c>
       <c r="H472" s="2" t="s">
         <v>1508</v>
@@ -25208,10 +25229,10 @@
         <v>942</v>
       </c>
       <c r="J472" s="2" t="s">
-        <v>1633</v>
+        <v>1640</v>
       </c>
       <c r="K472" s="2" t="s">
-        <v>1634</v>
+        <v>1641</v>
       </c>
       <c r="L472" s="2" t="s">
         <v>23</v>
@@ -25228,16 +25249,16 @@
         <v>14</v>
       </c>
       <c r="D473" s="2" t="s">
-        <v>1635</v>
+        <v>1642</v>
       </c>
       <c r="E473" s="2" t="s">
-        <v>1636</v>
+        <v>1643</v>
       </c>
       <c r="F473" s="2" t="s">
-        <v>1623</v>
+        <v>1630</v>
       </c>
       <c r="G473" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H473" s="2" t="s">
         <v>1508</v>
@@ -25246,10 +25267,10 @@
         <v>942</v>
       </c>
       <c r="J473" s="2" t="s">
-        <v>1637</v>
+        <v>1644</v>
       </c>
       <c r="K473" s="2" t="s">
-        <v>1638</v>
+        <v>1645</v>
       </c>
       <c r="L473" s="2" t="s">
         <v>23</v>
@@ -25266,16 +25287,16 @@
         <v>14</v>
       </c>
       <c r="D474" s="2" t="s">
-        <v>1639</v>
+        <v>1646</v>
       </c>
       <c r="E474" s="2" t="s">
-        <v>1640</v>
+        <v>1647</v>
       </c>
       <c r="F474" s="2" t="s">
-        <v>1623</v>
+        <v>1630</v>
       </c>
       <c r="G474" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H474" s="2" t="s">
         <v>1508</v>
@@ -25284,10 +25305,10 @@
         <v>942</v>
       </c>
       <c r="J474" s="2" t="s">
-        <v>1641</v>
+        <v>1648</v>
       </c>
       <c r="K474" s="2" t="s">
-        <v>1642</v>
+        <v>1649</v>
       </c>
       <c r="L474" s="2" t="s">
         <v>23</v>
@@ -25304,16 +25325,16 @@
         <v>14</v>
       </c>
       <c r="D475" s="2" t="s">
-        <v>1643</v>
+        <v>1650</v>
       </c>
       <c r="E475" s="2" t="s">
-        <v>1644</v>
+        <v>1651</v>
       </c>
       <c r="F475" s="2" t="s">
-        <v>1623</v>
+        <v>1630</v>
       </c>
       <c r="G475" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H475" s="2" t="s">
         <v>1508</v>
@@ -25322,10 +25343,10 @@
         <v>942</v>
       </c>
       <c r="J475" s="2" t="s">
-        <v>1645</v>
+        <v>1652</v>
       </c>
       <c r="K475" s="2" t="s">
-        <v>1646</v>
+        <v>1653</v>
       </c>
       <c r="L475" s="2" t="s">
         <v>23</v>
@@ -25342,28 +25363,28 @@
         <v>14</v>
       </c>
       <c r="D476" s="2" t="s">
-        <v>1647</v>
+        <v>1654</v>
       </c>
       <c r="E476" s="2" t="s">
-        <v>1648</v>
+        <v>1655</v>
       </c>
       <c r="F476" s="2" t="s">
-        <v>1623</v>
+        <v>1630</v>
       </c>
       <c r="G476" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H476" s="2" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="I476" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J476" s="2" t="s">
-        <v>1649</v>
+        <v>1656</v>
       </c>
       <c r="K476" s="2" t="s">
-        <v>1650</v>
+        <v>1657</v>
       </c>
       <c r="L476" s="2" t="s">
         <v>23</v>
@@ -25380,28 +25401,28 @@
         <v>14</v>
       </c>
       <c r="D477" s="2" t="s">
-        <v>1651</v>
+        <v>1658</v>
       </c>
       <c r="E477" s="2" t="s">
-        <v>1652</v>
+        <v>1659</v>
       </c>
       <c r="F477" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G477" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H477" s="2" t="s">
-        <v>1654</v>
+        <v>1661</v>
       </c>
       <c r="I477" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J477" s="2" t="s">
-        <v>1655</v>
+        <v>1662</v>
       </c>
       <c r="K477" s="2" t="s">
-        <v>1656</v>
+        <v>1663</v>
       </c>
       <c r="L477" s="2" t="s">
         <v>23</v>
@@ -25418,16 +25439,16 @@
         <v>14</v>
       </c>
       <c r="D478" s="2" t="s">
-        <v>1657</v>
+        <v>1664</v>
       </c>
       <c r="E478" s="2" t="s">
-        <v>1658</v>
+        <v>1665</v>
       </c>
       <c r="F478" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G478" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H478" s="2" t="s">
         <v>1508</v>
@@ -25436,10 +25457,10 @@
         <v>20</v>
       </c>
       <c r="J478" s="2" t="s">
-        <v>1659</v>
+        <v>1666</v>
       </c>
       <c r="K478" s="2" t="s">
-        <v>1660</v>
+        <v>1667</v>
       </c>
       <c r="L478" s="2" t="s">
         <v>23</v>
@@ -25456,16 +25477,16 @@
         <v>14</v>
       </c>
       <c r="D479" s="2" t="s">
-        <v>1661</v>
+        <v>1668</v>
       </c>
       <c r="E479" s="2" t="s">
-        <v>1662</v>
+        <v>1669</v>
       </c>
       <c r="F479" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G479" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H479" s="2" t="s">
         <v>1508</v>
@@ -25474,10 +25495,10 @@
         <v>20</v>
       </c>
       <c r="J479" s="2" t="s">
-        <v>1663</v>
+        <v>1670</v>
       </c>
       <c r="K479" s="2" t="s">
-        <v>1664</v>
+        <v>1671</v>
       </c>
       <c r="L479" s="2" t="s">
         <v>23</v>
@@ -25494,28 +25515,28 @@
         <v>14</v>
       </c>
       <c r="D480" s="2" t="s">
-        <v>1665</v>
+        <v>1672</v>
       </c>
       <c r="E480" s="2" t="s">
-        <v>1666</v>
+        <v>1673</v>
       </c>
       <c r="F480" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G480" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H480" s="2" t="s">
-        <v>1654</v>
+        <v>1661</v>
       </c>
       <c r="I480" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J480" s="2" t="s">
-        <v>1667</v>
+        <v>1674</v>
       </c>
       <c r="K480" s="2" t="s">
-        <v>1668</v>
+        <v>1675</v>
       </c>
       <c r="L480" s="2" t="s">
         <v>23</v>
@@ -25532,16 +25553,16 @@
         <v>14</v>
       </c>
       <c r="D481" s="2" t="s">
-        <v>1669</v>
+        <v>1676</v>
       </c>
       <c r="E481" s="2" t="s">
-        <v>1670</v>
+        <v>1677</v>
       </c>
       <c r="F481" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G481" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H481" s="2" t="s">
         <v>1508</v>
@@ -25550,10 +25571,10 @@
         <v>20</v>
       </c>
       <c r="J481" s="2" t="s">
-        <v>1671</v>
+        <v>1678</v>
       </c>
       <c r="K481" s="2" t="s">
-        <v>1672</v>
+        <v>1679</v>
       </c>
       <c r="L481" s="2" t="s">
         <v>23</v>
@@ -25570,28 +25591,28 @@
         <v>14</v>
       </c>
       <c r="D482" s="2" t="s">
-        <v>1673</v>
+        <v>1680</v>
       </c>
       <c r="E482" s="2" t="s">
-        <v>1674</v>
+        <v>1681</v>
       </c>
       <c r="F482" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G482" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H482" s="2" t="s">
-        <v>1654</v>
+        <v>1661</v>
       </c>
       <c r="I482" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J482" s="2" t="s">
-        <v>1663</v>
+        <v>1670</v>
       </c>
       <c r="K482" s="2" t="s">
-        <v>1675</v>
+        <v>1682</v>
       </c>
       <c r="L482" s="2" t="s">
         <v>23</v>
@@ -25608,16 +25629,16 @@
         <v>14</v>
       </c>
       <c r="D483" s="2" t="s">
-        <v>1676</v>
+        <v>1683</v>
       </c>
       <c r="E483" s="2" t="s">
-        <v>1677</v>
+        <v>1684</v>
       </c>
       <c r="F483" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G483" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H483" s="2" t="s">
         <v>1508</v>
@@ -25626,10 +25647,10 @@
         <v>20</v>
       </c>
       <c r="J483" s="2" t="s">
-        <v>1678</v>
+        <v>1685</v>
       </c>
       <c r="K483" s="2" t="s">
-        <v>1679</v>
+        <v>1686</v>
       </c>
       <c r="L483" s="2" t="s">
         <v>23</v>
@@ -25646,16 +25667,16 @@
         <v>14</v>
       </c>
       <c r="D484" s="2" t="s">
-        <v>1680</v>
+        <v>1687</v>
       </c>
       <c r="E484" s="2" t="s">
-        <v>1681</v>
+        <v>1688</v>
       </c>
       <c r="F484" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G484" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H484" s="2" t="s">
         <v>1508</v>
@@ -25664,10 +25685,10 @@
         <v>20</v>
       </c>
       <c r="J484" s="2" t="s">
-        <v>1682</v>
+        <v>1689</v>
       </c>
       <c r="K484" s="2" t="s">
-        <v>1683</v>
+        <v>1690</v>
       </c>
       <c r="L484" s="2" t="s">
         <v>23</v>
@@ -25684,28 +25705,28 @@
         <v>14</v>
       </c>
       <c r="D485" s="2" t="s">
-        <v>1684</v>
+        <v>1691</v>
       </c>
       <c r="E485" s="2" t="s">
+        <v>1692</v>
+      </c>
+      <c r="F485" s="2" t="s">
+        <v>1660</v>
+      </c>
+      <c r="G485" s="2" t="s">
+        <v>1631</v>
+      </c>
+      <c r="H485" s="2" t="s">
+        <v>1661</v>
+      </c>
+      <c r="I485" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J485" s="2" t="s">
         <v>1685</v>
       </c>
-      <c r="F485" s="2" t="s">
-        <v>1653</v>
-      </c>
-      <c r="G485" s="2" t="s">
-        <v>1624</v>
-      </c>
-      <c r="H485" s="2" t="s">
-        <v>1654</v>
-      </c>
-      <c r="I485" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J485" s="2" t="s">
-        <v>1678</v>
-      </c>
       <c r="K485" s="2" t="s">
-        <v>1686</v>
+        <v>1693</v>
       </c>
       <c r="L485" s="2" t="s">
         <v>23</v>
@@ -25722,28 +25743,28 @@
         <v>14</v>
       </c>
       <c r="D486" s="2" t="s">
-        <v>1687</v>
+        <v>1694</v>
       </c>
       <c r="E486" s="2" t="s">
-        <v>1688</v>
+        <v>1695</v>
       </c>
       <c r="F486" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G486" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H486" s="2" t="s">
-        <v>1689</v>
+        <v>1696</v>
       </c>
       <c r="I486" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J486" s="2" t="s">
-        <v>1690</v>
+        <v>1697</v>
       </c>
       <c r="K486" s="2" t="s">
-        <v>1691</v>
+        <v>1698</v>
       </c>
       <c r="L486" s="2" t="s">
         <v>23</v>
@@ -25760,28 +25781,28 @@
         <v>14</v>
       </c>
       <c r="D487" s="2" t="s">
-        <v>1692</v>
+        <v>1699</v>
       </c>
       <c r="E487" s="2" t="s">
-        <v>1693</v>
+        <v>1700</v>
       </c>
       <c r="F487" s="2" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="G487" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H487" s="2" t="s">
-        <v>1694</v>
+        <v>1701</v>
       </c>
       <c r="I487" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J487" s="2" t="s">
-        <v>1695</v>
+        <v>1702</v>
       </c>
       <c r="K487" s="2" t="s">
-        <v>1696</v>
+        <v>1703</v>
       </c>
       <c r="L487" s="2" t="s">
         <v>23</v>
@@ -25798,28 +25819,28 @@
         <v>14</v>
       </c>
       <c r="D488" s="2" t="s">
-        <v>1697</v>
+        <v>1704</v>
       </c>
       <c r="E488" s="2" t="s">
-        <v>1698</v>
+        <v>1705</v>
       </c>
       <c r="F488" s="2" t="s">
-        <v>1699</v>
+        <v>1706</v>
       </c>
       <c r="G488" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H488" s="2" t="s">
-        <v>1700</v>
+        <v>1707</v>
       </c>
       <c r="I488" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J488" s="2" t="s">
-        <v>1701</v>
+        <v>1708</v>
       </c>
       <c r="K488" s="2" t="s">
-        <v>1702</v>
+        <v>1709</v>
       </c>
       <c r="L488" s="2" t="s">
         <v>23</v>
@@ -25836,16 +25857,16 @@
         <v>14</v>
       </c>
       <c r="D489" s="2" t="s">
-        <v>1703</v>
+        <v>1710</v>
       </c>
       <c r="E489" s="2" t="s">
-        <v>1704</v>
+        <v>1711</v>
       </c>
       <c r="F489" s="2" t="s">
-        <v>1699</v>
+        <v>1706</v>
       </c>
       <c r="G489" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H489" s="2" t="s">
         <v>1508</v>
@@ -25854,10 +25875,10 @@
         <v>942</v>
       </c>
       <c r="J489" s="2" t="s">
-        <v>1705</v>
+        <v>1712</v>
       </c>
       <c r="K489" s="2" t="s">
-        <v>1706</v>
+        <v>1713</v>
       </c>
       <c r="L489" s="2" t="s">
         <v>23</v>
@@ -25874,16 +25895,16 @@
         <v>14</v>
       </c>
       <c r="D490" s="2" t="s">
-        <v>1707</v>
+        <v>1714</v>
       </c>
       <c r="E490" s="2" t="s">
-        <v>1708</v>
+        <v>1715</v>
       </c>
       <c r="F490" s="2" t="s">
-        <v>1699</v>
+        <v>1706</v>
       </c>
       <c r="G490" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H490" s="2" t="s">
         <v>1508</v>
@@ -25892,10 +25913,10 @@
         <v>942</v>
       </c>
       <c r="J490" s="2" t="s">
-        <v>1709</v>
+        <v>1716</v>
       </c>
       <c r="K490" s="2" t="s">
-        <v>1710</v>
+        <v>1717</v>
       </c>
       <c r="L490" s="2" t="s">
         <v>23</v>
@@ -25912,28 +25933,28 @@
         <v>14</v>
       </c>
       <c r="D491" s="2" t="s">
-        <v>1711</v>
+        <v>1718</v>
       </c>
       <c r="E491" s="2" t="s">
-        <v>1652</v>
+        <v>1659</v>
       </c>
       <c r="F491" s="2" t="s">
-        <v>1699</v>
+        <v>1706</v>
       </c>
       <c r="G491" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H491" s="2" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="I491" s="4" t="s">
         <v>942</v>
       </c>
       <c r="J491" s="2" t="s">
-        <v>1712</v>
+        <v>1719</v>
       </c>
       <c r="K491" s="2" t="s">
-        <v>1713</v>
+        <v>1720</v>
       </c>
       <c r="L491" s="2" t="s">
         <v>23</v>
@@ -25950,28 +25971,28 @@
         <v>14</v>
       </c>
       <c r="D492" s="2" t="s">
-        <v>1714</v>
+        <v>1721</v>
       </c>
       <c r="E492" s="2" t="s">
-        <v>1715</v>
+        <v>1722</v>
       </c>
       <c r="F492" s="2" t="s">
-        <v>1716</v>
+        <v>1723</v>
       </c>
       <c r="G492" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H492" s="2" t="s">
-        <v>1700</v>
+        <v>1707</v>
       </c>
       <c r="I492" s="4" t="s">
         <v>942</v>
       </c>
       <c r="J492" s="2" t="s">
-        <v>1717</v>
+        <v>1724</v>
       </c>
       <c r="K492" s="2" t="s">
-        <v>1718</v>
+        <v>1725</v>
       </c>
       <c r="L492" s="2" t="s">
         <v>23</v>
@@ -25988,16 +26009,16 @@
         <v>14</v>
       </c>
       <c r="D493" s="2" t="s">
-        <v>1719</v>
+        <v>1726</v>
       </c>
       <c r="E493" s="2" t="s">
-        <v>1704</v>
+        <v>1711</v>
       </c>
       <c r="F493" s="2" t="s">
-        <v>1716</v>
+        <v>1723</v>
       </c>
       <c r="G493" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H493" s="2" t="s">
         <v>1508</v>
@@ -26006,10 +26027,10 @@
         <v>20</v>
       </c>
       <c r="J493" s="2" t="s">
-        <v>1720</v>
+        <v>1727</v>
       </c>
       <c r="K493" s="2" t="s">
-        <v>1721</v>
+        <v>1728</v>
       </c>
       <c r="L493" s="2" t="s">
         <v>23</v>
@@ -26026,28 +26047,28 @@
         <v>14</v>
       </c>
       <c r="D494" s="2" t="s">
-        <v>1722</v>
+        <v>1729</v>
       </c>
       <c r="E494" s="2" t="s">
+        <v>1730</v>
+      </c>
+      <c r="F494" s="2" t="s">
         <v>1723</v>
       </c>
-      <c r="F494" s="2" t="s">
-        <v>1716</v>
-      </c>
       <c r="G494" s="2" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="H494" s="2" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="I494" s="4" t="s">
         <v>942</v>
       </c>
       <c r="J494" s="2" t="s">
-        <v>1724</v>
+        <v>1731</v>
       </c>
       <c r="K494" s="2" t="s">
-        <v>1725</v>
+        <v>1732</v>
       </c>
       <c r="L494" s="2" t="s">
         <v>23</v>
@@ -26064,13 +26085,13 @@
         <v>14</v>
       </c>
       <c r="D495" s="2" t="s">
-        <v>1726</v>
+        <v>1733</v>
       </c>
       <c r="E495" s="2" t="s">
-        <v>1727</v>
+        <v>1734</v>
       </c>
       <c r="F495" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G495" s="2" t="s">
         <v>1507</v>
@@ -26082,7 +26103,7 @@
         <v>1427</v>
       </c>
       <c r="J495" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K495" s="2" t="s">
         <v>23</v>
@@ -26102,13 +26123,13 @@
         <v>14</v>
       </c>
       <c r="D496" s="2" t="s">
-        <v>1730</v>
+        <v>1737</v>
       </c>
       <c r="E496" s="2" t="s">
-        <v>1731</v>
+        <v>1738</v>
       </c>
       <c r="F496" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G496" s="2" t="s">
         <v>1507</v>
@@ -26120,7 +26141,7 @@
         <v>1427</v>
       </c>
       <c r="J496" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K496" s="2" t="s">
         <v>23</v>
@@ -26140,13 +26161,13 @@
         <v>14</v>
       </c>
       <c r="D497" s="2" t="s">
-        <v>1732</v>
+        <v>1739</v>
       </c>
       <c r="E497" s="2" t="s">
-        <v>1733</v>
+        <v>1740</v>
       </c>
       <c r="F497" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G497" s="2" t="s">
         <v>1507</v>
@@ -26158,7 +26179,7 @@
         <v>1427</v>
       </c>
       <c r="J497" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K497" s="2" t="s">
         <v>23</v>
@@ -26178,13 +26199,13 @@
         <v>14</v>
       </c>
       <c r="D498" s="2" t="s">
-        <v>1734</v>
+        <v>1741</v>
       </c>
       <c r="E498" s="2" t="s">
+        <v>1742</v>
+      </c>
+      <c r="F498" s="2" t="s">
         <v>1735</v>
-      </c>
-      <c r="F498" s="2" t="s">
-        <v>1728</v>
       </c>
       <c r="G498" s="2" t="s">
         <v>1507</v>
@@ -26196,7 +26217,7 @@
         <v>1427</v>
       </c>
       <c r="J498" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K498" s="2" t="s">
         <v>23</v>
@@ -26216,13 +26237,13 @@
         <v>14</v>
       </c>
       <c r="D499" s="2" t="s">
-        <v>1736</v>
+        <v>1743</v>
       </c>
       <c r="E499" s="2" t="s">
-        <v>1737</v>
+        <v>1744</v>
       </c>
       <c r="F499" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G499" s="2" t="s">
         <v>1507</v>
@@ -26234,7 +26255,7 @@
         <v>1427</v>
       </c>
       <c r="J499" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K499" s="2" t="s">
         <v>23</v>
@@ -26254,13 +26275,13 @@
         <v>14</v>
       </c>
       <c r="D500" s="2" t="s">
-        <v>1738</v>
+        <v>1745</v>
       </c>
       <c r="E500" s="2" t="s">
-        <v>1739</v>
+        <v>1746</v>
       </c>
       <c r="F500" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G500" s="2" t="s">
         <v>1507</v>
@@ -26272,7 +26293,7 @@
         <v>1427</v>
       </c>
       <c r="J500" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K500" s="2" t="s">
         <v>23</v>
@@ -26292,13 +26313,13 @@
         <v>14</v>
       </c>
       <c r="D501" s="2" t="s">
-        <v>1740</v>
+        <v>1747</v>
       </c>
       <c r="E501" s="2" t="s">
-        <v>1741</v>
+        <v>1748</v>
       </c>
       <c r="F501" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G501" s="2" t="s">
         <v>1507</v>
@@ -26310,7 +26331,7 @@
         <v>1427</v>
       </c>
       <c r="J501" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K501" s="2" t="s">
         <v>23</v>
@@ -26330,13 +26351,13 @@
         <v>14</v>
       </c>
       <c r="D502" s="2" t="s">
-        <v>1742</v>
+        <v>1749</v>
       </c>
       <c r="E502" s="2" t="s">
-        <v>1743</v>
+        <v>1750</v>
       </c>
       <c r="F502" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G502" s="2" t="s">
         <v>1507</v>
@@ -26348,7 +26369,7 @@
         <v>1427</v>
       </c>
       <c r="J502" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K502" s="2" t="s">
         <v>23</v>
@@ -26368,13 +26389,13 @@
         <v>14</v>
       </c>
       <c r="D503" s="2" t="s">
-        <v>1744</v>
+        <v>1751</v>
       </c>
       <c r="E503" s="2" t="s">
-        <v>1745</v>
+        <v>1752</v>
       </c>
       <c r="F503" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G503" s="2" t="s">
         <v>1507</v>
@@ -26386,7 +26407,7 @@
         <v>1427</v>
       </c>
       <c r="J503" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K503" s="2" t="s">
         <v>23</v>
@@ -26406,13 +26427,13 @@
         <v>14</v>
       </c>
       <c r="D504" s="2" t="s">
-        <v>1746</v>
+        <v>1753</v>
       </c>
       <c r="E504" s="2" t="s">
-        <v>1747</v>
+        <v>1754</v>
       </c>
       <c r="F504" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G504" s="2" t="s">
         <v>1507</v>
@@ -26424,7 +26445,7 @@
         <v>1427</v>
       </c>
       <c r="J504" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K504" s="2" t="s">
         <v>23</v>
@@ -26444,13 +26465,13 @@
         <v>14</v>
       </c>
       <c r="D505" s="2" t="s">
-        <v>1748</v>
+        <v>1755</v>
       </c>
       <c r="E505" s="2" t="s">
-        <v>1749</v>
+        <v>1756</v>
       </c>
       <c r="F505" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G505" s="2" t="s">
         <v>1507</v>
@@ -26462,7 +26483,7 @@
         <v>1427</v>
       </c>
       <c r="J505" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K505" s="2" t="s">
         <v>23</v>
@@ -26482,13 +26503,13 @@
         <v>14</v>
       </c>
       <c r="D506" s="2" t="s">
-        <v>1750</v>
+        <v>1757</v>
       </c>
       <c r="E506" s="2" t="s">
-        <v>1751</v>
+        <v>1758</v>
       </c>
       <c r="F506" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G506" s="2" t="s">
         <v>1507</v>
@@ -26500,7 +26521,7 @@
         <v>1427</v>
       </c>
       <c r="J506" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K506" s="2" t="s">
         <v>23</v>
@@ -26520,13 +26541,13 @@
         <v>14</v>
       </c>
       <c r="D507" s="2" t="s">
-        <v>1752</v>
+        <v>1759</v>
       </c>
       <c r="E507" s="2" t="s">
-        <v>1753</v>
+        <v>1760</v>
       </c>
       <c r="F507" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G507" s="2" t="s">
         <v>1507</v>
@@ -26538,7 +26559,7 @@
         <v>1427</v>
       </c>
       <c r="J507" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K507" s="2" t="s">
         <v>23</v>
@@ -26558,13 +26579,13 @@
         <v>14</v>
       </c>
       <c r="D508" s="2" t="s">
-        <v>1754</v>
+        <v>1761</v>
       </c>
       <c r="E508" s="2" t="s">
-        <v>1755</v>
+        <v>1762</v>
       </c>
       <c r="F508" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G508" s="2" t="s">
         <v>1507</v>
@@ -26576,7 +26597,7 @@
         <v>1427</v>
       </c>
       <c r="J508" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K508" s="2" t="s">
         <v>23</v>
@@ -26596,13 +26617,13 @@
         <v>14</v>
       </c>
       <c r="D509" s="2" t="s">
-        <v>1756</v>
+        <v>1763</v>
       </c>
       <c r="E509" s="2" t="s">
-        <v>1757</v>
+        <v>1764</v>
       </c>
       <c r="F509" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G509" s="2" t="s">
         <v>1507</v>
@@ -26614,7 +26635,7 @@
         <v>1427</v>
       </c>
       <c r="J509" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K509" s="2" t="s">
         <v>23</v>
@@ -26634,13 +26655,13 @@
         <v>14</v>
       </c>
       <c r="D510" s="2" t="s">
-        <v>1758</v>
+        <v>1765</v>
       </c>
       <c r="E510" s="2" t="s">
-        <v>1759</v>
+        <v>1766</v>
       </c>
       <c r="F510" s="2" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="G510" s="2" t="s">
         <v>1507</v>
@@ -26652,7 +26673,7 @@
         <v>1427</v>
       </c>
       <c r="J510" s="2" t="s">
-        <v>1729</v>
+        <v>1736</v>
       </c>
       <c r="K510" s="2" t="s">
         <v>23</v>
@@ -26663,7 +26684,7 @@
     </row>
     <row r="511" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A511" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B511" s="2" t="s">
         <v>107</v>
@@ -26672,13 +26693,13 @@
         <v>14</v>
       </c>
       <c r="D511" s="2" t="s">
-        <v>1761</v>
+        <v>1768</v>
       </c>
       <c r="E511" s="2" t="s">
-        <v>1762</v>
+        <v>1769</v>
       </c>
       <c r="F511" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G511" s="2" t="s">
         <v>894</v>
@@ -26690,10 +26711,10 @@
         <v>20</v>
       </c>
       <c r="J511" s="2" t="s">
-        <v>1764</v>
+        <v>1771</v>
       </c>
       <c r="K511" s="2" t="s">
-        <v>1765</v>
+        <v>1772</v>
       </c>
       <c r="L511" s="2" t="s">
         <v>1099</v>
@@ -26701,7 +26722,7 @@
     </row>
     <row r="512" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A512" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B512" s="2" t="s">
         <v>107</v>
@@ -26710,13 +26731,13 @@
         <v>14</v>
       </c>
       <c r="D512" s="2" t="s">
-        <v>1766</v>
+        <v>1773</v>
       </c>
       <c r="E512" s="2" t="s">
-        <v>1767</v>
+        <v>1774</v>
       </c>
       <c r="F512" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G512" s="2" t="s">
         <v>894</v>
@@ -26728,10 +26749,10 @@
         <v>20</v>
       </c>
       <c r="J512" s="2" t="s">
-        <v>1768</v>
+        <v>1775</v>
       </c>
       <c r="K512" s="2" t="s">
-        <v>1769</v>
+        <v>1776</v>
       </c>
       <c r="L512" s="2" t="s">
         <v>1099</v>
@@ -26739,7 +26760,7 @@
     </row>
     <row r="513" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A513" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B513" s="2" t="s">
         <v>107</v>
@@ -26748,13 +26769,13 @@
         <v>14</v>
       </c>
       <c r="D513" s="2" t="s">
+        <v>1777</v>
+      </c>
+      <c r="E513" s="2" t="s">
+        <v>1778</v>
+      </c>
+      <c r="F513" s="2" t="s">
         <v>1770</v>
-      </c>
-      <c r="E513" s="2" t="s">
-        <v>1771</v>
-      </c>
-      <c r="F513" s="2" t="s">
-        <v>1763</v>
       </c>
       <c r="G513" s="2" t="s">
         <v>894</v>
@@ -26766,10 +26787,10 @@
         <v>20</v>
       </c>
       <c r="J513" s="2" t="s">
-        <v>1772</v>
+        <v>1779</v>
       </c>
       <c r="K513" s="2" t="s">
-        <v>1773</v>
+        <v>1780</v>
       </c>
       <c r="L513" s="2" t="s">
         <v>1099</v>
@@ -26777,7 +26798,7 @@
     </row>
     <row r="514" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A514" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B514" s="2" t="s">
         <v>107</v>
@@ -26786,13 +26807,13 @@
         <v>14</v>
       </c>
       <c r="D514" s="2" t="s">
-        <v>1774</v>
+        <v>1781</v>
       </c>
       <c r="E514" s="2" t="s">
-        <v>1775</v>
+        <v>1782</v>
       </c>
       <c r="F514" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G514" s="2" t="s">
         <v>894</v>
@@ -26804,10 +26825,10 @@
         <v>20</v>
       </c>
       <c r="J514" s="2" t="s">
-        <v>1776</v>
+        <v>1783</v>
       </c>
       <c r="K514" s="2" t="s">
-        <v>1777</v>
+        <v>1784</v>
       </c>
       <c r="L514" s="2" t="s">
         <v>1099</v>
@@ -26815,7 +26836,7 @@
     </row>
     <row r="515" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A515" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B515" s="2" t="s">
         <v>107</v>
@@ -26824,13 +26845,13 @@
         <v>14</v>
       </c>
       <c r="D515" s="2" t="s">
-        <v>1778</v>
+        <v>1785</v>
       </c>
       <c r="E515" s="2" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
       <c r="F515" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G515" s="2" t="s">
         <v>894</v>
@@ -26842,10 +26863,10 @@
         <v>20</v>
       </c>
       <c r="J515" s="2" t="s">
-        <v>1780</v>
+        <v>1787</v>
       </c>
       <c r="K515" s="2" t="s">
-        <v>1781</v>
+        <v>1788</v>
       </c>
       <c r="L515" s="2" t="s">
         <v>23</v>
@@ -26853,7 +26874,7 @@
     </row>
     <row r="516" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A516" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B516" s="2" t="s">
         <v>107</v>
@@ -26862,13 +26883,13 @@
         <v>14</v>
       </c>
       <c r="D516" s="2" t="s">
-        <v>1782</v>
+        <v>1789</v>
       </c>
       <c r="E516" s="2" t="s">
-        <v>1783</v>
+        <v>1790</v>
       </c>
       <c r="F516" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G516" s="2" t="s">
         <v>894</v>
@@ -26880,10 +26901,10 @@
         <v>20</v>
       </c>
       <c r="J516" s="2" t="s">
-        <v>1784</v>
+        <v>1791</v>
       </c>
       <c r="K516" s="2" t="s">
-        <v>1785</v>
+        <v>1792</v>
       </c>
       <c r="L516" s="2" t="s">
         <v>23</v>
@@ -26891,7 +26912,7 @@
     </row>
     <row r="517" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A517" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B517" s="2" t="s">
         <v>107</v>
@@ -26900,13 +26921,13 @@
         <v>14</v>
       </c>
       <c r="D517" s="2" t="s">
-        <v>1786</v>
+        <v>1793</v>
       </c>
       <c r="E517" s="2" t="s">
-        <v>1787</v>
+        <v>1794</v>
       </c>
       <c r="F517" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G517" s="2" t="s">
         <v>894</v>
@@ -26918,10 +26939,10 @@
         <v>20</v>
       </c>
       <c r="J517" s="2" t="s">
-        <v>1788</v>
+        <v>1795</v>
       </c>
       <c r="K517" s="2" t="s">
-        <v>1789</v>
+        <v>1796</v>
       </c>
       <c r="L517" s="2" t="s">
         <v>23</v>
@@ -26929,7 +26950,7 @@
     </row>
     <row r="518" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A518" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B518" s="2" t="s">
         <v>107</v>
@@ -26938,13 +26959,13 @@
         <v>14</v>
       </c>
       <c r="D518" s="2" t="s">
-        <v>1790</v>
+        <v>1797</v>
       </c>
       <c r="E518" s="2" t="s">
-        <v>1791</v>
+        <v>1798</v>
       </c>
       <c r="F518" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G518" s="2" t="s">
         <v>894</v>
@@ -26956,10 +26977,10 @@
         <v>20</v>
       </c>
       <c r="J518" s="2" t="s">
-        <v>1792</v>
+        <v>1799</v>
       </c>
       <c r="K518" s="2" t="s">
-        <v>1793</v>
+        <v>1800</v>
       </c>
       <c r="L518" s="2" t="s">
         <v>23</v>
@@ -26967,7 +26988,7 @@
     </row>
     <row r="519" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A519" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B519" s="2" t="s">
         <v>107</v>
@@ -26976,13 +26997,13 @@
         <v>14</v>
       </c>
       <c r="D519" s="2" t="s">
-        <v>1794</v>
+        <v>1801</v>
       </c>
       <c r="E519" s="2" t="s">
-        <v>1795</v>
+        <v>1802</v>
       </c>
       <c r="F519" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G519" s="2" t="s">
         <v>894</v>
@@ -26994,10 +27015,10 @@
         <v>20</v>
       </c>
       <c r="J519" s="2" t="s">
-        <v>1796</v>
+        <v>1803</v>
       </c>
       <c r="K519" s="2" t="s">
-        <v>1797</v>
+        <v>1804</v>
       </c>
       <c r="L519" s="2" t="s">
         <v>23</v>
@@ -27005,7 +27026,7 @@
     </row>
     <row r="520" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A520" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B520" s="2" t="s">
         <v>107</v>
@@ -27014,13 +27035,13 @@
         <v>14</v>
       </c>
       <c r="D520" s="2" t="s">
-        <v>1798</v>
+        <v>1805</v>
       </c>
       <c r="E520" s="2" t="s">
-        <v>1799</v>
+        <v>1806</v>
       </c>
       <c r="F520" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G520" s="2" t="s">
         <v>894</v>
@@ -27032,10 +27053,10 @@
         <v>20</v>
       </c>
       <c r="J520" s="2" t="s">
-        <v>1800</v>
+        <v>1807</v>
       </c>
       <c r="K520" s="2" t="s">
-        <v>1801</v>
+        <v>1808</v>
       </c>
       <c r="L520" s="2" t="s">
         <v>23</v>
@@ -27043,7 +27064,7 @@
     </row>
     <row r="521" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A521" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B521" s="2" t="s">
         <v>107</v>
@@ -27052,13 +27073,13 @@
         <v>14</v>
       </c>
       <c r="D521" s="2" t="s">
-        <v>1802</v>
+        <v>1809</v>
       </c>
       <c r="E521" s="2" t="s">
-        <v>1803</v>
+        <v>1810</v>
       </c>
       <c r="F521" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G521" s="2" t="s">
         <v>894</v>
@@ -27070,10 +27091,10 @@
         <v>20</v>
       </c>
       <c r="J521" s="2" t="s">
-        <v>1804</v>
+        <v>1811</v>
       </c>
       <c r="K521" s="2" t="s">
-        <v>1805</v>
+        <v>1812</v>
       </c>
       <c r="L521" s="2" t="s">
         <v>23</v>
@@ -27081,7 +27102,7 @@
     </row>
     <row r="522" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A522" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B522" s="2" t="s">
         <v>107</v>
@@ -27090,13 +27111,13 @@
         <v>14</v>
       </c>
       <c r="D522" s="2" t="s">
-        <v>1806</v>
+        <v>1813</v>
       </c>
       <c r="E522" s="2" t="s">
-        <v>1807</v>
+        <v>1814</v>
       </c>
       <c r="F522" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G522" s="2" t="s">
         <v>894</v>
@@ -27108,10 +27129,10 @@
         <v>20</v>
       </c>
       <c r="J522" s="2" t="s">
-        <v>1808</v>
+        <v>1815</v>
       </c>
       <c r="K522" s="2" t="s">
-        <v>1809</v>
+        <v>1816</v>
       </c>
       <c r="L522" s="2" t="s">
         <v>23</v>
@@ -27119,7 +27140,7 @@
     </row>
     <row r="523" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A523" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B523" s="2" t="s">
         <v>107</v>
@@ -27128,13 +27149,13 @@
         <v>14</v>
       </c>
       <c r="D523" s="2" t="s">
-        <v>1810</v>
+        <v>1817</v>
       </c>
       <c r="E523" s="2" t="s">
-        <v>1811</v>
+        <v>1818</v>
       </c>
       <c r="F523" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G523" s="2" t="s">
         <v>894</v>
@@ -27146,10 +27167,10 @@
         <v>20</v>
       </c>
       <c r="J523" s="2" t="s">
+        <v>1819</v>
+      </c>
+      <c r="K523" s="2" t="s">
         <v>1812</v>
-      </c>
-      <c r="K523" s="2" t="s">
-        <v>1805</v>
       </c>
       <c r="L523" s="2" t="s">
         <v>23</v>
@@ -27157,37 +27178,37 @@
     </row>
     <row r="524" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A524" s="2" t="s">
-        <v>1813</v>
+        <v>1820</v>
       </c>
       <c r="B524" s="2" t="s">
-        <v>1814</v>
+        <v>1821</v>
       </c>
       <c r="C524" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D524" s="2" t="s">
-        <v>1815</v>
+        <v>1822</v>
       </c>
       <c r="E524" s="2" t="s">
-        <v>1816</v>
+        <v>1823</v>
       </c>
       <c r="F524" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G524" s="2" t="s">
         <v>894</v>
       </c>
       <c r="H524" s="2" t="s">
-        <v>1817</v>
+        <v>1824</v>
       </c>
       <c r="I524" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J524" s="2" t="s">
-        <v>1818</v>
+        <v>1825</v>
       </c>
       <c r="K524" s="2" t="s">
-        <v>1819</v>
+        <v>1826</v>
       </c>
       <c r="L524" s="2" t="s">
         <v>616</v>
@@ -27195,37 +27216,37 @@
     </row>
     <row r="525" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A525" s="2" t="s">
-        <v>1813</v>
+        <v>1820</v>
       </c>
       <c r="B525" s="2" t="s">
-        <v>1814</v>
+        <v>1821</v>
       </c>
       <c r="C525" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D525" s="2" t="s">
-        <v>1820</v>
+        <v>1827</v>
       </c>
       <c r="E525" s="2" t="s">
-        <v>1821</v>
+        <v>1828</v>
       </c>
       <c r="F525" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G525" s="2" t="s">
         <v>894</v>
       </c>
       <c r="H525" s="2" t="s">
-        <v>1817</v>
+        <v>1824</v>
       </c>
       <c r="I525" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J525" s="2" t="s">
-        <v>1822</v>
+        <v>1829</v>
       </c>
       <c r="K525" s="2" t="s">
-        <v>1823</v>
+        <v>1830</v>
       </c>
       <c r="L525" s="2" t="s">
         <v>616</v>
@@ -27233,37 +27254,37 @@
     </row>
     <row r="526" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A526" s="2" t="s">
-        <v>1813</v>
+        <v>1820</v>
       </c>
       <c r="B526" s="2" t="s">
-        <v>1814</v>
+        <v>1821</v>
       </c>
       <c r="C526" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D526" s="2" t="s">
-        <v>1824</v>
+        <v>1831</v>
       </c>
       <c r="E526" s="2" t="s">
-        <v>1825</v>
+        <v>1832</v>
       </c>
       <c r="F526" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G526" s="2" t="s">
         <v>894</v>
       </c>
       <c r="H526" s="2" t="s">
-        <v>1817</v>
+        <v>1824</v>
       </c>
       <c r="I526" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J526" s="2" t="s">
-        <v>1826</v>
+        <v>1833</v>
       </c>
       <c r="K526" s="2" t="s">
-        <v>1827</v>
+        <v>1834</v>
       </c>
       <c r="L526" s="2" t="s">
         <v>616</v>
@@ -27271,37 +27292,37 @@
     </row>
     <row r="527" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A527" s="2" t="s">
-        <v>1813</v>
+        <v>1820</v>
       </c>
       <c r="B527" s="2" t="s">
-        <v>1814</v>
+        <v>1821</v>
       </c>
       <c r="C527" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D527" s="2" t="s">
-        <v>1828</v>
+        <v>1835</v>
       </c>
       <c r="E527" s="2" t="s">
-        <v>1829</v>
+        <v>1836</v>
       </c>
       <c r="F527" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G527" s="2" t="s">
         <v>894</v>
       </c>
       <c r="H527" s="2" t="s">
-        <v>1817</v>
+        <v>1824</v>
       </c>
       <c r="I527" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J527" s="2" t="s">
-        <v>1830</v>
+        <v>1837</v>
       </c>
       <c r="K527" s="2" t="s">
-        <v>1831</v>
+        <v>1838</v>
       </c>
       <c r="L527" s="2" t="s">
         <v>616</v>
@@ -27309,37 +27330,37 @@
     </row>
     <row r="528" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A528" s="2" t="s">
-        <v>1813</v>
+        <v>1820</v>
       </c>
       <c r="B528" s="2" t="s">
-        <v>1814</v>
+        <v>1821</v>
       </c>
       <c r="C528" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D528" s="2" t="s">
-        <v>1832</v>
+        <v>1839</v>
       </c>
       <c r="E528" s="2" t="s">
-        <v>1833</v>
+        <v>1840</v>
       </c>
       <c r="F528" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G528" s="2" t="s">
         <v>894</v>
       </c>
       <c r="H528" s="2" t="s">
-        <v>1817</v>
+        <v>1824</v>
       </c>
       <c r="I528" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J528" s="2" t="s">
-        <v>1834</v>
+        <v>1841</v>
       </c>
       <c r="K528" s="2" t="s">
-        <v>1835</v>
+        <v>1842</v>
       </c>
       <c r="L528" s="2" t="s">
         <v>616</v>
@@ -27347,37 +27368,37 @@
     </row>
     <row r="529" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A529" s="2" t="s">
-        <v>1813</v>
+        <v>1820</v>
       </c>
       <c r="B529" s="2" t="s">
-        <v>1814</v>
+        <v>1821</v>
       </c>
       <c r="C529" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D529" s="2" t="s">
-        <v>1836</v>
+        <v>1843</v>
       </c>
       <c r="E529" s="2" t="s">
-        <v>1837</v>
+        <v>1844</v>
       </c>
       <c r="F529" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G529" s="2" t="s">
         <v>894</v>
       </c>
       <c r="H529" s="2" t="s">
-        <v>1817</v>
+        <v>1824</v>
       </c>
       <c r="I529" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J529" s="2" t="s">
-        <v>1838</v>
+        <v>1845</v>
       </c>
       <c r="K529" s="2" t="s">
-        <v>1839</v>
+        <v>1846</v>
       </c>
       <c r="L529" s="2" t="s">
         <v>616</v>
@@ -27385,37 +27406,37 @@
     </row>
     <row r="530" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A530" s="2" t="s">
-        <v>1813</v>
+        <v>1820</v>
       </c>
       <c r="B530" s="2" t="s">
-        <v>1814</v>
+        <v>1821</v>
       </c>
       <c r="C530" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D530" s="2" t="s">
-        <v>1840</v>
+        <v>1847</v>
       </c>
       <c r="E530" s="2" t="s">
-        <v>1841</v>
+        <v>1848</v>
       </c>
       <c r="F530" s="2" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="G530" s="2" t="s">
         <v>894</v>
       </c>
       <c r="H530" s="2" t="s">
-        <v>1817</v>
+        <v>1824</v>
       </c>
       <c r="I530" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J530" s="2" t="s">
-        <v>1842</v>
+        <v>1849</v>
       </c>
       <c r="K530" s="2" t="s">
-        <v>1843</v>
+        <v>1850</v>
       </c>
       <c r="L530" s="2" t="s">
         <v>616</v>
@@ -27448,51 +27469,51 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>1844</v>
+        <v>1851</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1845</v>
+        <v>1852</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1846</v>
+        <v>1853</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1847</v>
+        <v>1854</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1848</v>
+        <v>1855</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1849</v>
+        <v>1856</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1850</v>
+        <v>1857</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>1851</v>
+        <v>1858</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>1852</v>
+        <v>1859</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>1853</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="2" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>1854</v>
+        <v>1861</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1856</v>
+        <v>1863</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>123</v>
@@ -27510,27 +27531,27 @@
         <v>4</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>1857</v>
+        <v>1864</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>1858</v>
+        <v>1865</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>1860</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>1861</v>
+        <v>1868</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1862</v>
+        <v>1869</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>123</v>
@@ -27548,27 +27569,27 @@
         <v>4</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>1857</v>
+        <v>1864</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>1858</v>
+        <v>1865</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>1860</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>1863</v>
+        <v>1870</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1864</v>
+        <v>1871</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>123</v>
@@ -27586,27 +27607,27 @@
         <v>4</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>1857</v>
+        <v>1864</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>1858</v>
+        <v>1865</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>1860</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="5" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>1865</v>
+        <v>1872</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1866</v>
+        <v>1873</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>123</v>
@@ -27624,27 +27645,27 @@
         <v>4</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>1857</v>
+        <v>1864</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>1858</v>
+        <v>1865</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>1860</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="6" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>1867</v>
+        <v>1874</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1868</v>
+        <v>1875</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>141</v>
@@ -27662,27 +27683,27 @@
         <v>3</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>1869</v>
+        <v>1876</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>1870</v>
+        <v>1877</v>
       </c>
     </row>
     <row r="7" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>1871</v>
+        <v>1878</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1872</v>
+        <v>1879</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>141</v>
@@ -27700,27 +27721,27 @@
         <v>3</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>1869</v>
+        <v>1876</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>1870</v>
+        <v>1877</v>
       </c>
     </row>
     <row r="8" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>1873</v>
+        <v>1880</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1874</v>
+        <v>1881</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>74</v>
@@ -27738,27 +27759,27 @@
         <v>4</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>1875</v>
+        <v>1882</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>1575</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>1876</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="9" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>1877</v>
+        <v>1884</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1878</v>
+        <v>1885</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>74</v>
@@ -27776,16 +27797,16 @@
         <v>4</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>1875</v>
+        <v>1882</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>1575</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>1876</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -27793,10 +27814,10 @@
         <v>106</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1879</v>
+        <v>1886</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>107</v>
@@ -27814,27 +27835,27 @@
         <v>1</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>1880</v>
+        <v>1887</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>1881</v>
+        <v>1888</v>
       </c>
     </row>
     <row r="11" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>1882</v>
+        <v>1889</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1883</v>
+        <v>1890</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>190</v>
@@ -27852,27 +27873,27 @@
         <v>2</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>1884</v>
+        <v>1891</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>616</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>1885</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="12" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>1886</v>
+        <v>1893</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1887</v>
+        <v>1894</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>190</v>
@@ -27890,27 +27911,27 @@
         <v>2</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>1884</v>
+        <v>1891</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>616</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>1885</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="13" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>1888</v>
+        <v>1895</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1889</v>
+        <v>1896</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>13</v>
@@ -27928,27 +27949,27 @@
         <v>2</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>1880</v>
+        <v>1887</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>616</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>1890</v>
+        <v>1897</v>
       </c>
     </row>
     <row r="14" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>1891</v>
+        <v>1898</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1855</v>
+        <v>1862</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1892</v>
+        <v>1899</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>13</v>
@@ -27966,16 +27987,16 @@
         <v>2</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>1880</v>
+        <v>1887</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>616</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>1890</v>
+        <v>1897</v>
       </c>
     </row>
     <row r="15" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -27983,10 +28004,10 @@
         <v>828</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1893</v>
+        <v>1900</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1894</v>
+        <v>1901</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>141</v>
@@ -28004,16 +28025,16 @@
         <v>0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>1895</v>
+        <v>1902</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>1896</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="16" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -28021,10 +28042,10 @@
         <v>810</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1893</v>
+        <v>1900</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1897</v>
+        <v>1904</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>74</v>
@@ -28042,16 +28063,16 @@
         <v>0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>1895</v>
+        <v>1902</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>1898</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="17" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -28059,10 +28080,10 @@
         <v>542</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>1893</v>
+        <v>1900</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>1899</v>
+        <v>1906</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>123</v>
@@ -28080,16 +28101,16 @@
         <v>0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>1895</v>
+        <v>1902</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>1900</v>
+        <v>1907</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>1901</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="18" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -28097,10 +28118,10 @@
         <v>805</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1893</v>
+        <v>1900</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1902</v>
+        <v>1909</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>123</v>
@@ -28118,16 +28139,16 @@
         <v>0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>1895</v>
+        <v>1902</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>897</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>1903</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="19" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -28135,10 +28156,10 @@
         <v>833</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>1893</v>
+        <v>1900</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>1904</v>
+        <v>1911</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>123</v>
@@ -28156,16 +28177,16 @@
         <v>0</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>1895</v>
+        <v>1902</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>1905</v>
+        <v>1912</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>1906</v>
+        <v>1913</v>
       </c>
     </row>
     <row r="20" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -28173,10 +28194,10 @@
         <v>730</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>1907</v>
+        <v>1914</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1908</v>
+        <v>1915</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>190</v>
@@ -28194,16 +28215,16 @@
         <v>0</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>1909</v>
+        <v>1916</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>1910</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="21" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -28211,10 +28232,10 @@
         <v>1108</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>1911</v>
+        <v>1918</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>1912</v>
+        <v>1919</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>13</v>
@@ -28232,16 +28253,16 @@
         <v>0</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>1913</v>
+        <v>1920</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>1914</v>
+        <v>1921</v>
       </c>
     </row>
     <row r="22" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -28249,10 +28270,10 @@
         <v>845</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1915</v>
+        <v>1922</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1916</v>
+        <v>1923</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>141</v>
@@ -28270,16 +28291,16 @@
         <v>0</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>1917</v>
+        <v>1924</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>1918</v>
+        <v>1925</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>1919</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="23" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -28287,10 +28308,10 @@
         <v>1358</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>1920</v>
+        <v>1927</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>1921</v>
+        <v>1928</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>141</v>
@@ -28308,27 +28329,27 @@
         <v>4</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>1922</v>
+        <v>1929</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>1923</v>
+        <v>1930</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>1924</v>
+        <v>1931</v>
       </c>
     </row>
     <row r="24" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1925</v>
+        <v>1932</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1926</v>
+        <v>1933</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>107</v>
@@ -28346,16 +28367,16 @@
         <v>0</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>1927</v>
+        <v>1934</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>1099</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>1859</v>
+        <v>1866</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>1928</v>
+        <v>1935</v>
       </c>
     </row>
   </sheetData>
@@ -28383,60 +28404,60 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>1929</v>
+        <v>1936</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1930</v>
+        <v>1937</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1931</v>
+        <v>1938</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1846</v>
+        <v>1853</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1847</v>
+        <v>1854</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1848</v>
+        <v>1855</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1932</v>
+        <v>1939</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>1933</v>
+        <v>1940</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>1934</v>
+        <v>1941</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>1935</v>
+        <v>1942</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>1851</v>
+        <v>1858</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>1936</v>
+        <v>1943</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1937</v>
+        <v>1944</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1938</v>
+        <v>1945</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>1939</v>
+        <v>1946</v>
       </c>
       <c r="F2" s="2">
         <v>138</v>
@@ -28457,27 +28478,27 @@
         <v>86</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>1940</v>
+        <v>1947</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>1941</v>
+        <v>1948</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>1942</v>
+        <v>1949</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1943</v>
+        <v>1950</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1944</v>
+        <v>1951</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>1945</v>
+        <v>1952</v>
       </c>
       <c r="F3" s="2">
         <v>120</v>
@@ -28498,27 +28519,27 @@
         <v>17</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>1946</v>
+        <v>1953</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>1947</v>
+        <v>1954</v>
       </c>
     </row>
     <row r="4" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>1948</v>
+        <v>1955</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1949</v>
+        <v>1956</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1950</v>
+        <v>1957</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1951</v>
+        <v>1958</v>
       </c>
       <c r="F4" s="2">
         <v>87</v>
@@ -28539,7 +28560,7 @@
         <v>41</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>1952</v>
+        <v>1959</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>1575</v>
@@ -28547,19 +28568,19 @@
     </row>
     <row r="5" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>1953</v>
+        <v>1960</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1954</v>
+        <v>1961</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1955</v>
+        <v>1962</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1956</v>
+        <v>1963</v>
       </c>
       <c r="F5" s="2">
         <v>55</v>
@@ -28580,7 +28601,7 @@
         <v>19</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>1957</v>
+        <v>1964</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>1099</v>
@@ -28588,19 +28609,19 @@
     </row>
     <row r="6" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>1958</v>
+        <v>1965</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1959</v>
+        <v>1966</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1960</v>
+        <v>1967</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1961</v>
+        <v>1968</v>
       </c>
       <c r="F6" s="2">
         <v>56</v>
@@ -28621,7 +28642,7 @@
         <v>21</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>1962</v>
+        <v>1969</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>616</v>
@@ -28629,19 +28650,19 @@
     </row>
     <row r="7" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>1963</v>
+        <v>1970</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1964</v>
+        <v>1971</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1965</v>
+        <v>1972</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1966</v>
+        <v>1973</v>
       </c>
       <c r="F7" s="2">
         <v>66</v>
@@ -28662,7 +28683,7 @@
         <v>35</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>1967</v>
+        <v>1974</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>616</v>
@@ -28691,31 +28712,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>1968</v>
+        <v>1975</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>1969</v>
+        <v>1976</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>1846</v>
+        <v>1853</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>1847</v>
+        <v>1854</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>1848</v>
+        <v>1855</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>1849</v>
+        <v>1856</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>1970</v>
+        <v>1977</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>1971</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -28723,7 +28744,7 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>1972</v>
+        <v>1979</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -28741,10 +28762,10 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>1973</v>
+        <v>1980</v>
       </c>
       <c r="I2" t="s">
-        <v>1974</v>
+        <v>1981</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -28752,7 +28773,7 @@
         <v>325</v>
       </c>
       <c r="B3" t="s">
-        <v>1975</v>
+        <v>1982</v>
       </c>
       <c r="C3" t="s">
         <v>326</v>
@@ -28770,10 +28791,10 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>1976</v>
+        <v>1983</v>
       </c>
       <c r="I3" t="s">
-        <v>1977</v>
+        <v>1984</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -28781,7 +28802,7 @@
         <v>893</v>
       </c>
       <c r="B4" t="s">
-        <v>1978</v>
+        <v>1985</v>
       </c>
       <c r="C4" t="s">
         <v>894</v>
@@ -28799,10 +28820,10 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>1979</v>
+        <v>1986</v>
       </c>
       <c r="I4" t="s">
-        <v>1980</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -28810,7 +28831,7 @@
         <v>1111</v>
       </c>
       <c r="B5" t="s">
-        <v>1981</v>
+        <v>1988</v>
       </c>
       <c r="C5" t="s">
         <v>894</v>
@@ -28828,10 +28849,10 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>1982</v>
+        <v>1989</v>
       </c>
       <c r="I5" t="s">
-        <v>1983</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -28839,7 +28860,7 @@
         <v>1136</v>
       </c>
       <c r="B6" t="s">
-        <v>1984</v>
+        <v>1991</v>
       </c>
       <c r="C6" t="s">
         <v>894</v>
@@ -28857,10 +28878,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>1985</v>
+        <v>1992</v>
       </c>
       <c r="I6" t="s">
-        <v>1986</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -28868,7 +28889,7 @@
         <v>1506</v>
       </c>
       <c r="B7" t="s">
-        <v>1987</v>
+        <v>1994</v>
       </c>
       <c r="C7" t="s">
         <v>1507</v>
@@ -28886,18 +28907,18 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>1988</v>
+        <v>1995</v>
       </c>
       <c r="I7" t="s">
-        <v>1989</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="B8" t="s">
-        <v>1990</v>
+        <v>1997</v>
       </c>
       <c r="C8" t="s">
         <v>1507</v>
@@ -28915,21 +28936,21 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>1991</v>
+        <v>1998</v>
       </c>
       <c r="I8" t="s">
-        <v>1992</v>
+        <v>1999</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1623</v>
+        <v>1630</v>
       </c>
       <c r="B9" t="s">
-        <v>1993</v>
+        <v>2000</v>
       </c>
       <c r="C9" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="D9">
         <v>7</v>
@@ -28944,21 +28965,21 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>1994</v>
+        <v>2001</v>
       </c>
       <c r="I9" t="s">
-        <v>1995</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>1653</v>
+        <v>1660</v>
       </c>
       <c r="B10" t="s">
-        <v>1996</v>
+        <v>2003</v>
       </c>
       <c r="C10" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="D10">
         <v>11</v>
@@ -28973,21 +28994,21 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>1997</v>
+        <v>2004</v>
       </c>
       <c r="I10" t="s">
-        <v>1998</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1699</v>
+        <v>1706</v>
       </c>
       <c r="B11" t="s">
-        <v>1999</v>
+        <v>2006</v>
       </c>
       <c r="C11" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="D11">
         <v>4</v>
@@ -29002,21 +29023,21 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>2000</v>
+        <v>2007</v>
       </c>
       <c r="I11" t="s">
-        <v>2001</v>
+        <v>2008</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>1716</v>
+        <v>1723</v>
       </c>
       <c r="B12" t="s">
-        <v>2002</v>
+        <v>2009</v>
       </c>
       <c r="C12" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
       <c r="D12">
         <v>3</v>
@@ -29031,18 +29052,18 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>2003</v>
+        <v>2010</v>
       </c>
       <c r="I12" t="s">
-        <v>2004</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="B13" t="s">
-        <v>2005</v>
+        <v>2012</v>
       </c>
       <c r="C13" t="s">
         <v>1507</v>
@@ -29060,18 +29081,18 @@
         <v>16</v>
       </c>
       <c r="H13" t="s">
-        <v>2006</v>
+        <v>2013</v>
       </c>
       <c r="I13" t="s">
-        <v>2007</v>
+        <v>2014</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>1763</v>
+        <v>1770</v>
       </c>
       <c r="B14" t="s">
-        <v>2008</v>
+        <v>2015</v>
       </c>
       <c r="C14" t="s">
         <v>894</v>
@@ -29089,10 +29110,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>2009</v>
+        <v>2016</v>
       </c>
       <c r="I14" t="s">
-        <v>2010</v>
+        <v>2017</v>
       </c>
     </row>
   </sheetData>
@@ -29117,25 +29138,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>1929</v>
+        <v>1936</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2011</v>
+        <v>2018</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2013</v>
+        <v>2020</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2014</v>
+        <v>2021</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>2015</v>
+        <v>2022</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>2016</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29143,68 +29164,68 @@
         <v>1363</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>2017</v>
+        <v>2024</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2018</v>
+        <v>2025</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>2020</v>
+        <v>2027</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>2021</v>
+        <v>2028</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>2023</v>
+        <v>2030</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>2024</v>
+        <v>2031</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>2025</v>
+        <v>2032</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>2026</v>
+        <v>2033</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>2027</v>
+        <v>2034</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>2028</v>
+        <v>2035</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>2036</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2037</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>2038</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>2039</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>2029</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>2030</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>2031</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>2032</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>2022</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29212,68 +29233,68 @@
         <v>1070</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>2033</v>
+        <v>2040</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>2034</v>
+        <v>2041</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>2035</v>
+        <v>2042</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>2036</v>
+        <v>2043</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>2037</v>
+        <v>2044</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>2038</v>
+        <v>2045</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>2039</v>
+        <v>2046</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>2034</v>
+        <v>2041</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>2040</v>
+        <v>2047</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>2041</v>
+        <v>2048</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>2042</v>
+        <v>2049</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>2043</v>
+        <v>2050</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>2044</v>
+        <v>2051</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>2034</v>
+        <v>2041</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>2045</v>
+        <v>2052</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>2046</v>
+        <v>2053</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>2042</v>
+        <v>2049</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29281,68 +29302,68 @@
         <v>1017</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>2047</v>
+        <v>2054</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>2048</v>
+        <v>2055</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>2049</v>
+        <v>2056</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>2050</v>
+        <v>2057</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>2051</v>
+        <v>2058</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>2052</v>
+        <v>2059</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>2053</v>
+        <v>2060</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>2054</v>
+        <v>2061</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>2055</v>
+        <v>2062</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>2056</v>
+        <v>2063</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>2057</v>
+        <v>2064</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>2058</v>
+        <v>2065</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>2059</v>
+        <v>2066</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>2060</v>
+        <v>2067</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>936</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>2042</v>
+        <v>2049</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29350,45 +29371,45 @@
         <v>329</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>2061</v>
+        <v>2068</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>2062</v>
+        <v>2069</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>2063</v>
+        <v>2070</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>2064</v>
+        <v>2071</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>2065</v>
+        <v>2072</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>2066</v>
+        <v>2073</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>2067</v>
+        <v>2074</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>2054</v>
+        <v>2061</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>2068</v>
+        <v>2075</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>2069</v>
+        <v>2076</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>2070</v>
+        <v>2077</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29396,45 +29417,45 @@
         <v>1099</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>2071</v>
+        <v>2078</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>2072</v>
+        <v>2079</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>2073</v>
+        <v>2080</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>2074</v>
+        <v>2081</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>2075</v>
+        <v>2082</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>2076</v>
+        <v>2083</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>2077</v>
+        <v>2084</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>2078</v>
+        <v>2085</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>2079</v>
+        <v>2086</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>2080</v>
+        <v>2087</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29442,22 +29463,22 @@
         <v>547</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>2081</v>
+        <v>2088</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>2082</v>
+        <v>2089</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>2083</v>
+        <v>2090</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>548</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>2084</v>
+        <v>2091</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29465,13 +29486,13 @@
         <v>1575</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>2085</v>
+        <v>2092</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>2086</v>
+        <v>2093</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>2087</v>
+        <v>2094</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>1571</v>
@@ -29480,7 +29501,7 @@
         <v>1571</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29488,22 +29509,22 @@
         <v>616</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>2088</v>
+        <v>2095</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>2089</v>
+        <v>2096</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>2090</v>
+        <v>2097</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>2091</v>
+        <v>2098</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>2092</v>
+        <v>2099</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29511,22 +29532,22 @@
         <v>1139</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>2093</v>
+        <v>2100</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>2094</v>
+        <v>2101</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>2095</v>
+        <v>2102</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>2096</v>
+        <v>2103</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>2097</v>
+        <v>2104</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -29534,68 +29555,68 @@
         <v>1228</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>2098</v>
+        <v>2105</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>2099</v>
+        <v>2106</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>2100</v>
+        <v>2107</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>1253</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>2101</v>
+        <v>2108</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>2102</v>
+        <v>2109</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>2103</v>
+        <v>2110</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>2104</v>
+        <v>2111</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>2105</v>
+        <v>2112</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>2106</v>
+        <v>2113</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="21" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>2107</v>
+        <v>2114</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>2108</v>
+        <v>2115</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>2109</v>
+        <v>2116</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>2110</v>
+        <v>2117</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>2111</v>
+        <v>2118</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>2022</v>
+        <v>2029</v>
       </c>
     </row>
   </sheetData>

</xml_diff>